<commit_message>
colocar relatorio 'separar' e gera tudo sobre os adultos
</commit_message>
<xml_diff>
--- a/PrestadorAdulto/neotin/resultado/relatorio_final.xlsx
+++ b/PrestadorAdulto/neotin/resultado/relatorio_final.xlsx
@@ -1199,31 +1199,31 @@
         <v>0</v>
       </c>
       <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" t="n">
         <v>2</v>
       </c>
-      <c r="F18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" t="n">
-        <v>5</v>
-      </c>
-      <c r="I18" t="n">
+      <c r="L18" t="n">
         <v>3</v>
       </c>
-      <c r="J18" t="n">
-        <v>0</v>
-      </c>
-      <c r="K18" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" t="n">
-        <v>0</v>
-      </c>
       <c r="M18" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -1233,40 +1233,40 @@
         </is>
       </c>
       <c r="B19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
+        <v>11</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="n">
+        <v>4</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" t="n">
         <v>3</v>
       </c>
-      <c r="C19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" t="n">
+      <c r="L19" t="n">
+        <v>3</v>
+      </c>
+      <c r="M19" t="n">
         <v>2</v>
-      </c>
-      <c r="F19" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" t="n">
-        <v>3</v>
-      </c>
-      <c r="I19" t="n">
-        <v>2</v>
-      </c>
-      <c r="J19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K19" t="n">
-        <v>1</v>
-      </c>
-      <c r="L19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M19" t="n">
-        <v>8</v>
       </c>
     </row>
     <row r="20">
@@ -1276,7 +1276,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C20" t="n">
         <v>0</v>
@@ -1291,19 +1291,19 @@
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H20" t="n">
         <v>0</v>
       </c>
       <c r="I20" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
       </c>
       <c r="K20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L20" t="n">
         <v>0</v>
@@ -1334,25 +1334,25 @@
         <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H21" t="n">
         <v>0</v>
       </c>
       <c r="I21" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L21" t="n">
         <v>0</v>
       </c>
       <c r="M21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -1377,7 +1377,7 @@
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H22" t="n">
         <v>0</v>
@@ -1395,7 +1395,7 @@
         <v>0</v>
       </c>
       <c r="M22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -1448,7 +1448,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C24" t="n">
         <v>0</v>
@@ -1463,19 +1463,19 @@
         <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="H24" t="n">
         <v>0</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
       </c>
       <c r="K24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L24" t="n">
         <v>0</v>
@@ -1586,7 +1586,7 @@
         <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F27" t="n">
         <v>0</v>
@@ -1595,19 +1595,19 @@
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" t="n">
         <v>2</v>
       </c>
-      <c r="J27" t="n">
-        <v>0</v>
-      </c>
-      <c r="K27" t="n">
-        <v>0</v>
-      </c>
       <c r="L27" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M27" t="n">
         <v>0</v>
@@ -1629,7 +1629,7 @@
         <v>0</v>
       </c>
       <c r="E28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F28" t="n">
         <v>0</v>
@@ -1696,7 +1696,7 @@
         <v>0</v>
       </c>
       <c r="M29" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -1724,7 +1724,7 @@
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I30" t="n">
         <v>0</v>
@@ -1801,7 +1801,7 @@
         <v>0</v>
       </c>
       <c r="E32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F32" t="n">
         <v>0</v>
@@ -1810,7 +1810,7 @@
         <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I32" t="n">
         <v>0</v>
@@ -1825,7 +1825,7 @@
         <v>0</v>
       </c>
       <c r="M32" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -2108,7 +2108,7 @@
         <v>0</v>
       </c>
       <c r="G39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H39" t="n">
         <v>0</v>
@@ -2292,7 +2292,7 @@
         <v>0</v>
       </c>
       <c r="K43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L43" t="n">
         <v>0</v>
@@ -2372,7 +2372,7 @@
         <v>0</v>
       </c>
       <c r="I45" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J45" t="n">
         <v>0</v>
@@ -2384,7 +2384,7 @@
         <v>0</v>
       </c>
       <c r="M45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46">
@@ -2452,7 +2452,7 @@
         <v>0</v>
       </c>
       <c r="G47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H47" t="n">
         <v>0</v>
@@ -2470,7 +2470,7 @@
         <v>0</v>
       </c>
       <c r="M47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">
@@ -2910,7 +2910,7 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="C58" t="n">
         <v>0</v>
@@ -2919,31 +2919,31 @@
         <v>0</v>
       </c>
       <c r="E58" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="F58" t="n">
         <v>0</v>
       </c>
       <c r="G58" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="H58" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="I58" t="n">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="J58" t="n">
         <v>0</v>
       </c>
       <c r="K58" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="L58" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="M58" t="n">
-        <v>28</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>